<commit_message>
feat: add original language description to Variables table (#6355)
* add field

* add field

* add field to docs

* add field to demodata

* add demodata

* bump version

* add version doc

---------

Co-authored-by: BHijmans <b.s.hijmans@umcg.nl>
Co-authored-by: Morris Swertz <m.a.swertz@rug.nl>
</commit_message>
<xml_diff>
--- a/docs/resources/Dictionary.xlsx
+++ b/docs/resources/Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brend\Molgenis\repos\molgenis-emx2\docs\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HijmansBS\Molgenis\repos\molgenis-emx2\docs\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB5D145-FCA1-4EB1-A4D5-355F1EC7BF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025ED455-6EED-4D3C-81D1-59D2344906EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15" yWindow="15" windowWidth="19185" windowHeight="11985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datasets" sheetId="9" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t>label</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>variable</t>
+  </si>
+  <si>
+    <t>original language description</t>
   </si>
 </sst>
 </file>
@@ -478,21 +481,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.06640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.9296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -531,31 +534,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:T1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.06640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.9296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.9296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.73046875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.1328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.19921875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="24.1328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.109375" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -572,48 +576,51 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>16</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>17</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>19</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>20</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>21</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>7</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>23</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>24</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>25</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -625,21 +632,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.59765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.53125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.46484375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.9296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
feat: add Variables.ontology term uri (#6430)
* add demo data
* ontology termURI to hyperlink
* versioning
* edit docs
* edit templates
</commit_message>
<xml_diff>
--- a/docs/resources/Dictionary.xlsx
+++ b/docs/resources/Dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HijmansBS\Molgenis\repos\molgenis-emx2\docs\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025ED455-6EED-4D3C-81D1-59D2344906EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB159B3-E296-42B6-A020-5FF7E2CF9ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>label</t>
   </si>
@@ -534,32 +534,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="27.88671875" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="24.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -588,39 +589,42 @@
         <v>17</v>
       </c>
       <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>18</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>19</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>20</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>21</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>22</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>23</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>24</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>25</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rename table Datasets to Tables (#6416)
</commit_message>
<xml_diff>
--- a/docs/resources/Dictionary.xlsx
+++ b/docs/resources/Dictionary.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HijmansBS\Molgenis\repos\molgenis-emx2\docs\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB159B3-E296-42B6-A020-5FF7E2CF9ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0393A85D-710D-4015-A7A0-C8CAC6F3075C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Datasets" sheetId="9" r:id="rId1"/>
+    <sheet name="Tables" sheetId="9" r:id="rId1"/>
     <sheet name="Variables" sheetId="13" r:id="rId2"/>
     <sheet name="Variable values" sheetId="20" r:id="rId3"/>
   </sheets>
@@ -39,9 +39,6 @@
     <t>order</t>
   </si>
   <si>
-    <t>dataset type</t>
-  </si>
-  <si>
     <t>unit of observation</t>
   </si>
   <si>
@@ -66,9 +63,6 @@
     <t>ontology term URI</t>
   </si>
   <si>
-    <t>dataset</t>
-  </si>
-  <si>
     <t>collection event</t>
   </si>
   <si>
@@ -99,9 +93,6 @@
     <t>useExternalDefinition.resource</t>
   </si>
   <si>
-    <t>useExternalDefinition.dataset</t>
-  </si>
-  <si>
     <t>useExternalDefinition.name</t>
   </si>
   <si>
@@ -109,6 +100,15 @@
   </si>
   <si>
     <t>original language description</t>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>useExternalDefinition.table</t>
+  </si>
+  <si>
+    <t>table type</t>
   </si>
 </sst>
 </file>
@@ -506,25 +506,25 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
-      </c>
-      <c r="J1" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -539,10 +539,10 @@
   <cols>
     <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="27.88671875" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" customWidth="1"/>
+    <col min="4" max="4" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
@@ -565,7 +565,7 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
         <v>3</v>
@@ -577,55 +577,55 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" t="s">
         <v>16</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
         <v>17</v>
       </c>
-      <c r="J1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>18</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>19</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
+        <v>6</v>
+      </c>
+      <c r="R1" t="s">
         <v>20</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" t="s">
-        <v>7</v>
-      </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>22</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" t="s">
         <v>23</v>
-      </c>
-      <c r="T1" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" t="s">
-        <v>25</v>
-      </c>
-      <c r="V1" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -638,10 +638,10 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
@@ -655,13 +655,13 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -670,16 +670,16 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" t="s">
-        <v>13</v>
-      </c>
       <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
         <v>9</v>
-      </c>
-      <c r="J1" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>